<commit_message>
Refactor duration handling from minutes to days across various scripts and tests
- Updated duration fields in CSV and JSON import/export scripts to use days instead of minutes.
- Adjusted related tests to reflect the change in duration units.
- Modified feasibility checker to account for capacity constraints and task incompatibilities.
- Enhanced documentation to clarify the changes in duration handling.
</commit_message>
<xml_diff>
--- a/Front/prismatron-solver-forge/public/gabarits/gabarit_ingestion_trco.xlsx
+++ b/Front/prismatron-solver-forge/public/gabarits/gabarit_ingestion_trco.xlsx
@@ -306,7 +306,7 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Durée en minutes pour CE couple tâche-ressource précisément (nombre entier positif).</t>
+        <t>Durée en jours pour CE couple tâche-ressource précisément (nombre entier positif).</t>
       </text>
     </comment>
   </commentList>
@@ -7009,7 +7009,7 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>duree_minutes *</t>
+          <t>duree_jours *</t>
         </is>
       </c>
     </row>
@@ -7025,11 +7025,11 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>← exemple : T1 prend 30 min sur M1</t>
+          <t>← exemple : T1 prend 3 jours sur R1</t>
         </is>
       </c>
     </row>
@@ -9531,7 +9531,7 @@
     <dataValidation sqref="B3:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Doit être un id déclaré dans l'onglet Ressources." type="list">
       <formula1>='Ressources'!$A$2:$A$500</formula1>
     </dataValidation>
-    <dataValidation sqref="C3:C500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="La durée doit être un nombre entier positif (en minutes)." type="whole" operator="greaterThan">
+    <dataValidation sqref="C3:C500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="La durée doit être un nombre entier positif (en jours)." type="whole" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>